<commit_message>
Updated POL_grids_kan10 model - 2026-06-30 21:03
</commit_message>
<xml_diff>
--- a/VerveStacks_POL_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_POL_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_POL_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D32EEE3C-5331-4654-AF4E-D57A7B058738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B73CB704-167C-4B6C-A358-8C0FA312740B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5827" uniqueCount="598">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5750" uniqueCount="577">
   <si>
     <t>Unit</t>
   </si>
@@ -1228,60 +1228,39 @@
     <t>grid_node</t>
   </si>
   <si>
-    <t>p_w139452056-400_POL</t>
-  </si>
-  <si>
-    <t>p_w183945016-220_POL</t>
-  </si>
-  <si>
-    <t>p_w255277953-400_POL</t>
-  </si>
-  <si>
-    <t>p_w44389929-220_POL</t>
+    <t>p_w29115701-220_POL</t>
+  </si>
+  <si>
+    <t>p_w39428977-400_POL</t>
+  </si>
+  <si>
+    <t>p_w86494356-400_POL</t>
+  </si>
+  <si>
+    <t>p_w111615226-220_POL</t>
+  </si>
+  <si>
+    <t>p_w133537926-220_POL</t>
+  </si>
+  <si>
+    <t>p_w191035265-220_POL</t>
+  </si>
+  <si>
+    <t>p_w293484891-220_POL</t>
+  </si>
+  <si>
+    <t>p_PL75-220_POL</t>
+  </si>
+  <si>
+    <t>p_PL17-400_POL</t>
   </si>
   <si>
     <t>p_w303870256-400_POL</t>
   </si>
   <si>
-    <t>p_w29115701-220_POL</t>
-  </si>
-  <si>
-    <t>p_w39428977-400_POL</t>
-  </si>
-  <si>
-    <t>p_w86494356-400_POL</t>
-  </si>
-  <si>
-    <t>p_w111615226-220_POL</t>
-  </si>
-  <si>
-    <t>p_w133537926-220_POL</t>
-  </si>
-  <si>
-    <t>p_w191035265-220_POL</t>
-  </si>
-  <si>
-    <t>p_w293484891-220_POL</t>
-  </si>
-  <si>
-    <t>p_PL75-220_POL</t>
-  </si>
-  <si>
-    <t>p_PL17-400_POL</t>
-  </si>
-  <si>
     <t>p_w255314292_POL</t>
   </si>
   <si>
-    <t>p_w166838338-400_POL</t>
-  </si>
-  <si>
-    <t>p_w173613665-220_POL</t>
-  </si>
-  <si>
-    <t>p_w215282393-400_POL</t>
-  </si>
-  <si>
     <t>rez_spv_POL_001</t>
   </si>
   <si>
@@ -1435,21 +1414,21 @@
     <t>admin_1</t>
   </si>
   <si>
+    <t>Makroregion województwo mazowieckie</t>
+  </si>
+  <si>
+    <t>Makroregion północno-zachodni</t>
+  </si>
+  <si>
+    <t>Makroregion północny</t>
+  </si>
+  <si>
+    <t>Makroregion południowo-zachodni</t>
+  </si>
+  <si>
     <t>Makroregion południowy</t>
   </si>
   <si>
-    <t>Makroregion południowo-zachodni</t>
-  </si>
-  <si>
-    <t>Makroregion północny</t>
-  </si>
-  <si>
-    <t>Makroregion województwo mazowieckie</t>
-  </si>
-  <si>
-    <t>Makroregion północno-zachodni</t>
-  </si>
-  <si>
     <t>Makroregion centralny</t>
   </si>
   <si>
@@ -1462,60 +1441,39 @@
     <t>region_com</t>
   </si>
   <si>
-    <t>e_w139452056-400_POL</t>
-  </si>
-  <si>
-    <t>e_w183945016-220_POL</t>
-  </si>
-  <si>
-    <t>e_w255277953-400_POL</t>
-  </si>
-  <si>
-    <t>e_w44389929-220_POL</t>
+    <t>e_w29115701-220_POL</t>
+  </si>
+  <si>
+    <t>e_w39428977-400_POL</t>
+  </si>
+  <si>
+    <t>e_w86494356-400_POL</t>
+  </si>
+  <si>
+    <t>e_w111615226-220_POL</t>
+  </si>
+  <si>
+    <t>e_w133537926-220_POL</t>
+  </si>
+  <si>
+    <t>e_w191035265-220_POL</t>
+  </si>
+  <si>
+    <t>e_w293484891-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL75-220_POL</t>
+  </si>
+  <si>
+    <t>e_PL17-400_POL</t>
   </si>
   <si>
     <t>e_w303870256-400_POL</t>
   </si>
   <si>
-    <t>e_w29115701-220_POL</t>
-  </si>
-  <si>
-    <t>e_w39428977-400_POL</t>
-  </si>
-  <si>
-    <t>e_w86494356-400_POL</t>
-  </si>
-  <si>
-    <t>e_w111615226-220_POL</t>
-  </si>
-  <si>
-    <t>e_w133537926-220_POL</t>
-  </si>
-  <si>
-    <t>e_w191035265-220_POL</t>
-  </si>
-  <si>
-    <t>e_w293484891-220_POL</t>
-  </si>
-  <si>
-    <t>e_PL75-220_POL</t>
-  </si>
-  <si>
-    <t>e_PL17-400_POL</t>
-  </si>
-  <si>
     <t>e_w255314292_POL</t>
   </si>
   <si>
-    <t>e_w166838338-400_POL</t>
-  </si>
-  <si>
-    <t>e_w173613665-220_POL</t>
-  </si>
-  <si>
-    <t>e_w215282393-400_POL</t>
-  </si>
-  <si>
     <t>elc_spv_POL_001</t>
   </si>
   <si>
@@ -1675,58 +1633,37 @@
     <t>lng</t>
   </si>
   <si>
-    <t>POL-e_w139452056-400_POL</t>
-  </si>
-  <si>
-    <t>POL-e_w183945016-220_POL</t>
-  </si>
-  <si>
-    <t>POL-e_w255277953-400_POL</t>
-  </si>
-  <si>
-    <t>POL-e_w44389929-220_POL</t>
+    <t>POL-e_w29115701-220_POL</t>
+  </si>
+  <si>
+    <t>POL-e_w39428977-400_POL</t>
+  </si>
+  <si>
+    <t>POL-e_w86494356-400_POL</t>
+  </si>
+  <si>
+    <t>POL-e_w111615226-220_POL</t>
+  </si>
+  <si>
+    <t>POL-e_w133537926-220_POL</t>
+  </si>
+  <si>
+    <t>POL-e_w191035265-220_POL</t>
+  </si>
+  <si>
+    <t>POL-e_w293484891-220_POL</t>
+  </si>
+  <si>
+    <t>POL-e_PL75-220_POL</t>
+  </si>
+  <si>
+    <t>POL-e_PL17-400_POL</t>
   </si>
   <si>
     <t>POL-e_w303870256-400_POL</t>
   </si>
   <si>
-    <t>POL-e_w29115701-220_POL</t>
-  </si>
-  <si>
-    <t>POL-e_w39428977-400_POL</t>
-  </si>
-  <si>
-    <t>POL-e_w86494356-400_POL</t>
-  </si>
-  <si>
-    <t>POL-e_w111615226-220_POL</t>
-  </si>
-  <si>
-    <t>POL-e_w133537926-220_POL</t>
-  </si>
-  <si>
-    <t>POL-e_w191035265-220_POL</t>
-  </si>
-  <si>
-    <t>POL-e_w293484891-220_POL</t>
-  </si>
-  <si>
-    <t>POL-e_PL75-220_POL</t>
-  </si>
-  <si>
-    <t>POL-e_PL17-400_POL</t>
-  </si>
-  <si>
     <t>POL-e_w255314292_POL</t>
-  </si>
-  <si>
-    <t>POL-e_w166838338-400_POL</t>
-  </si>
-  <si>
-    <t>POL-e_w173613665-220_POL</t>
-  </si>
-  <si>
-    <t>POL-e_w215282393-400_POL</t>
   </si>
   <si>
     <t>POL-elc_spv_POL_001</t>
@@ -22949,16 +22886,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4117FDD7-9430-417A-84A7-AFC76CA252B3}">
-  <dimension ref="B9:H78"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B73B8572-050C-405C-9660-642A7EE57C10}">
+  <dimension ref="B9:H71"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:8">
       <c r="B9" t="s">
-        <v>527</v>
+        <v>513</v>
       </c>
       <c r="F9" t="s">
-        <v>527</v>
+        <v>513</v>
       </c>
     </row>
     <row r="10" spans="2:8">
@@ -22966,19 +22903,19 @@
         <v>373</v>
       </c>
       <c r="C10" t="s">
-        <v>528</v>
+        <v>514</v>
       </c>
       <c r="D10" t="s">
-        <v>529</v>
+        <v>515</v>
       </c>
       <c r="F10" t="s">
         <v>373</v>
       </c>
       <c r="G10" t="s">
-        <v>528</v>
+        <v>514</v>
       </c>
       <c r="H10" t="s">
-        <v>529</v>
+        <v>515</v>
       </c>
     </row>
     <row r="11" spans="2:8">
@@ -22986,19 +22923,19 @@
         <v>381</v>
       </c>
       <c r="C11">
-        <v>50.123096251445361</v>
+        <v>52.214439540966481</v>
       </c>
       <c r="D11">
-        <v>18.541202951404959</v>
+        <v>20.877296701170323</v>
       </c>
       <c r="F11" t="s">
-        <v>530</v>
+        <v>516</v>
       </c>
       <c r="G11">
-        <v>50.123096251445361</v>
+        <v>52.214439540966481</v>
       </c>
       <c r="H11">
-        <v>18.541202951404959</v>
+        <v>20.877296701170323</v>
       </c>
     </row>
     <row r="12" spans="2:8">
@@ -23006,19 +22943,19 @@
         <v>382</v>
       </c>
       <c r="C12">
-        <v>50.130601442155474</v>
+        <v>53.196124772846453</v>
       </c>
       <c r="D12">
-        <v>18.849567300984408</v>
+        <v>14.476073038134793</v>
       </c>
       <c r="F12" t="s">
-        <v>531</v>
+        <v>517</v>
       </c>
       <c r="G12">
-        <v>50.130601442155474</v>
+        <v>53.196124772846453</v>
       </c>
       <c r="H12">
-        <v>18.849567300984408</v>
+        <v>14.476073038134793</v>
       </c>
     </row>
     <row r="13" spans="2:8">
@@ -23026,19 +22963,19 @@
         <v>383</v>
       </c>
       <c r="C13">
-        <v>50.746544696597532</v>
+        <v>54.718832956325642</v>
       </c>
       <c r="D13">
-        <v>17.872695321486159</v>
+        <v>18.109334026299528</v>
       </c>
       <c r="F13" t="s">
-        <v>532</v>
+        <v>518</v>
       </c>
       <c r="G13">
-        <v>50.746544696597532</v>
+        <v>54.718832956325642</v>
       </c>
       <c r="H13">
-        <v>17.872695321486159</v>
+        <v>18.109334026299528</v>
       </c>
     </row>
     <row r="14" spans="2:8">
@@ -23046,19 +22983,19 @@
         <v>384</v>
       </c>
       <c r="C14">
-        <v>49.84240724566758</v>
+        <v>51.092587962369954</v>
       </c>
       <c r="D14">
-        <v>19.212740275249061</v>
+        <v>15.114048637999918</v>
       </c>
       <c r="F14" t="s">
-        <v>533</v>
+        <v>519</v>
       </c>
       <c r="G14">
-        <v>49.84240724566758</v>
+        <v>51.092587962369954</v>
       </c>
       <c r="H14">
-        <v>19.212740275249061</v>
+        <v>15.114048637999918</v>
       </c>
     </row>
     <row r="15" spans="2:8">
@@ -23066,19 +23003,19 @@
         <v>385</v>
       </c>
       <c r="C15">
-        <v>53.757586946292747</v>
+        <v>50.163695089947211</v>
       </c>
       <c r="D15">
-        <v>22.30185788377095</v>
+        <v>19.29195378291049</v>
       </c>
       <c r="F15" t="s">
-        <v>534</v>
+        <v>520</v>
       </c>
       <c r="G15">
-        <v>53.757586946292747</v>
+        <v>50.163695089947211</v>
       </c>
       <c r="H15">
-        <v>22.30185788377095</v>
+        <v>19.29195378291049</v>
       </c>
     </row>
     <row r="16" spans="2:8">
@@ -23086,19 +23023,19 @@
         <v>386</v>
       </c>
       <c r="C16">
-        <v>52.214439540966481</v>
+        <v>50.063820992731642</v>
       </c>
       <c r="D16">
-        <v>20.877296701170323</v>
+        <v>20.944770681767888</v>
       </c>
       <c r="F16" t="s">
-        <v>535</v>
+        <v>521</v>
       </c>
       <c r="G16">
-        <v>52.214439540966481</v>
+        <v>50.063820992731642</v>
       </c>
       <c r="H16">
-        <v>20.877296701170323</v>
+        <v>20.944770681767888</v>
       </c>
     </row>
     <row r="17" spans="2:8">
@@ -23106,19 +23043,19 @@
         <v>387</v>
       </c>
       <c r="C17">
-        <v>53.196124772846453</v>
+        <v>51.316035643998099</v>
       </c>
       <c r="D17">
-        <v>14.476073038134793</v>
+        <v>19.328367738135</v>
       </c>
       <c r="F17" t="s">
-        <v>536</v>
+        <v>522</v>
       </c>
       <c r="G17">
-        <v>53.196124772846453</v>
+        <v>51.316035643998099</v>
       </c>
       <c r="H17">
-        <v>14.476073038134793</v>
+        <v>19.328367738135</v>
       </c>
     </row>
     <row r="18" spans="2:8">
@@ -23126,19 +23063,19 @@
         <v>388</v>
       </c>
       <c r="C18">
-        <v>54.718832956325642</v>
+        <v>49.888401941940245</v>
       </c>
       <c r="D18">
-        <v>18.109334026299528</v>
+        <v>18.690068508639264</v>
       </c>
       <c r="F18" t="s">
-        <v>537</v>
+        <v>523</v>
       </c>
       <c r="G18">
-        <v>54.718832956325642</v>
+        <v>49.888401941940245</v>
       </c>
       <c r="H18">
-        <v>18.109334026299528</v>
+        <v>18.690068508639264</v>
       </c>
     </row>
     <row r="19" spans="2:8">
@@ -23146,19 +23083,19 @@
         <v>389</v>
       </c>
       <c r="C19">
-        <v>51.092587962369954</v>
+        <v>52.9345914951098</v>
       </c>
       <c r="D19">
-        <v>15.114048637999918</v>
+        <v>22.9435906</v>
       </c>
       <c r="F19" t="s">
-        <v>538</v>
+        <v>524</v>
       </c>
       <c r="G19">
-        <v>51.092587962369954</v>
+        <v>52.9345914951098</v>
       </c>
       <c r="H19">
-        <v>15.114048637999918</v>
+        <v>22.9435906</v>
       </c>
     </row>
     <row r="20" spans="2:8">
@@ -23166,19 +23103,19 @@
         <v>390</v>
       </c>
       <c r="C20">
-        <v>50.163695089947211</v>
+        <v>53.757586946292747</v>
       </c>
       <c r="D20">
-        <v>19.29195378291049</v>
+        <v>22.30185788377095</v>
       </c>
       <c r="F20" t="s">
-        <v>539</v>
+        <v>525</v>
       </c>
       <c r="G20">
-        <v>50.163695089947211</v>
+        <v>53.757586946292747</v>
       </c>
       <c r="H20">
-        <v>19.29195378291049</v>
+        <v>22.30185788377095</v>
       </c>
     </row>
     <row r="21" spans="2:8">
@@ -23186,19 +23123,19 @@
         <v>391</v>
       </c>
       <c r="C21">
-        <v>50.063820992731642</v>
+        <v>54.502152608471313</v>
       </c>
       <c r="D21">
-        <v>20.944770681767888</v>
+        <v>16.89038355962467</v>
       </c>
       <c r="F21" t="s">
-        <v>540</v>
+        <v>526</v>
       </c>
       <c r="G21">
-        <v>50.063820992731642</v>
+        <v>54.502152608471313</v>
       </c>
       <c r="H21">
-        <v>20.944770681767888</v>
+        <v>16.89038355962467</v>
       </c>
     </row>
     <row r="22" spans="2:8">
@@ -23206,19 +23143,19 @@
         <v>392</v>
       </c>
       <c r="C22">
-        <v>51.316035643998099</v>
+        <v>51.583436367597201</v>
       </c>
       <c r="D22">
-        <v>19.328367738135</v>
+        <v>14.918750384776654</v>
       </c>
       <c r="F22" t="s">
-        <v>541</v>
+        <v>527</v>
       </c>
       <c r="G22">
-        <v>51.316035643998099</v>
+        <v>51.583436367597201</v>
       </c>
       <c r="H22">
-        <v>19.328367738135</v>
+        <v>14.918750384776654</v>
       </c>
     </row>
     <row r="23" spans="2:8">
@@ -23226,19 +23163,19 @@
         <v>393</v>
       </c>
       <c r="C23">
-        <v>49.888401941940245</v>
+        <v>50.345189363482064</v>
       </c>
       <c r="D23">
-        <v>18.690068508639264</v>
+        <v>17.419694531519191</v>
       </c>
       <c r="F23" t="s">
-        <v>542</v>
+        <v>528</v>
       </c>
       <c r="G23">
-        <v>49.888401941940245</v>
+        <v>50.345189363482064</v>
       </c>
       <c r="H23">
-        <v>18.690068508639264</v>
+        <v>17.419694531519191</v>
       </c>
     </row>
     <row r="24" spans="2:8">
@@ -23246,19 +23183,19 @@
         <v>394</v>
       </c>
       <c r="C24">
-        <v>52.9345914951098</v>
+        <v>51.394042753969877</v>
       </c>
       <c r="D24">
-        <v>22.9435906</v>
+        <v>16.751959330113646</v>
       </c>
       <c r="F24" t="s">
-        <v>543</v>
+        <v>529</v>
       </c>
       <c r="G24">
-        <v>52.9345914951098</v>
+        <v>51.394042753969877</v>
       </c>
       <c r="H24">
-        <v>22.9435906</v>
+        <v>16.751959330113646</v>
       </c>
     </row>
     <row r="25" spans="2:8">
@@ -23266,19 +23203,19 @@
         <v>395</v>
       </c>
       <c r="C25">
-        <v>54.502152608471313</v>
+        <v>52.622736475773067</v>
       </c>
       <c r="D25">
-        <v>16.89038355962467</v>
+        <v>14.990153475277031</v>
       </c>
       <c r="F25" t="s">
-        <v>544</v>
+        <v>530</v>
       </c>
       <c r="G25">
-        <v>54.502152608471313</v>
+        <v>52.622736475773067</v>
       </c>
       <c r="H25">
-        <v>16.89038355962467</v>
+        <v>14.990153475277031</v>
       </c>
     </row>
     <row r="26" spans="2:8">
@@ -23286,19 +23223,19 @@
         <v>396</v>
       </c>
       <c r="C26">
-        <v>49.688226064614483</v>
+        <v>52.928251230696389</v>
       </c>
       <c r="D26">
-        <v>21.852623292646182</v>
+        <v>16.824637442608388</v>
       </c>
       <c r="F26" t="s">
-        <v>545</v>
+        <v>531</v>
       </c>
       <c r="G26">
-        <v>49.688226064614483</v>
+        <v>52.928251230696389</v>
       </c>
       <c r="H26">
-        <v>21.852623292646182</v>
+        <v>16.824637442608388</v>
       </c>
     </row>
     <row r="27" spans="2:8">
@@ -23306,19 +23243,19 @@
         <v>397</v>
       </c>
       <c r="C27">
-        <v>50.716735959213132</v>
+        <v>54.059169587861376</v>
       </c>
       <c r="D27">
-        <v>23.292570654205857</v>
+        <v>20.643266624036407</v>
       </c>
       <c r="F27" t="s">
-        <v>546</v>
+        <v>532</v>
       </c>
       <c r="G27">
-        <v>50.716735959213132</v>
+        <v>54.059169587861376</v>
       </c>
       <c r="H27">
-        <v>23.292570654205857</v>
+        <v>20.643266624036407</v>
       </c>
     </row>
     <row r="28" spans="2:8">
@@ -23326,19 +23263,19 @@
         <v>398</v>
       </c>
       <c r="C28">
-        <v>50.190926527507919</v>
+        <v>54.160621229584443</v>
       </c>
       <c r="D28">
-        <v>21.87079962455832</v>
+        <v>16.92764152265681</v>
       </c>
       <c r="F28" t="s">
-        <v>547</v>
+        <v>533</v>
       </c>
       <c r="G28">
-        <v>50.190926527507919</v>
+        <v>54.160621229584443</v>
       </c>
       <c r="H28">
-        <v>21.87079962455832</v>
+        <v>16.92764152265681</v>
       </c>
     </row>
     <row r="29" spans="2:8">
@@ -23346,19 +23283,19 @@
         <v>399</v>
       </c>
       <c r="C29">
-        <v>51.583436367597201</v>
+        <v>53.850966420117743</v>
       </c>
       <c r="D29">
-        <v>14.918750384776654</v>
+        <v>19.007446557812909</v>
       </c>
       <c r="F29" t="s">
-        <v>548</v>
+        <v>534</v>
       </c>
       <c r="G29">
-        <v>51.583436367597201</v>
+        <v>53.850966420117743</v>
       </c>
       <c r="H29">
-        <v>14.918750384776654</v>
+        <v>19.007446557812909</v>
       </c>
     </row>
     <row r="30" spans="2:8">
@@ -23366,19 +23303,19 @@
         <v>400</v>
       </c>
       <c r="C30">
-        <v>50.345189363482064</v>
+        <v>52.430848156657824</v>
       </c>
       <c r="D30">
-        <v>17.419694531519191</v>
+        <v>23.043264145360411</v>
       </c>
       <c r="F30" t="s">
-        <v>549</v>
+        <v>535</v>
       </c>
       <c r="G30">
-        <v>50.345189363482064</v>
+        <v>52.430848156657824</v>
       </c>
       <c r="H30">
-        <v>17.419694531519191</v>
+        <v>23.043264145360411</v>
       </c>
     </row>
     <row r="31" spans="2:8">
@@ -23386,19 +23323,19 @@
         <v>401</v>
       </c>
       <c r="C31">
-        <v>51.394042753969877</v>
+        <v>54.306478182754368</v>
       </c>
       <c r="D31">
-        <v>16.751959330113646</v>
+        <v>22.2025648456056</v>
       </c>
       <c r="F31" t="s">
-        <v>550</v>
+        <v>536</v>
       </c>
       <c r="G31">
-        <v>51.394042753969877</v>
+        <v>54.306478182754368</v>
       </c>
       <c r="H31">
-        <v>16.751959330113646</v>
+        <v>22.2025648456056</v>
       </c>
     </row>
     <row r="32" spans="2:8">
@@ -23406,19 +23343,19 @@
         <v>402</v>
       </c>
       <c r="C32">
-        <v>52.622736475773067</v>
+        <v>53.408286508261966</v>
       </c>
       <c r="D32">
-        <v>14.990153475277031</v>
+        <v>22.619231503504921</v>
       </c>
       <c r="F32" t="s">
-        <v>551</v>
+        <v>537</v>
       </c>
       <c r="G32">
-        <v>52.622736475773067</v>
+        <v>53.408286508261966</v>
       </c>
       <c r="H32">
-        <v>14.990153475277031</v>
+        <v>22.619231503504921</v>
       </c>
     </row>
     <row r="33" spans="2:8">
@@ -23426,19 +23363,19 @@
         <v>403</v>
       </c>
       <c r="C33">
-        <v>52.928251230696389</v>
+        <v>49.725566374889411</v>
       </c>
       <c r="D33">
-        <v>16.824637442608388</v>
+        <v>22.73628524706481</v>
       </c>
       <c r="F33" t="s">
-        <v>552</v>
+        <v>538</v>
       </c>
       <c r="G33">
-        <v>52.928251230696389</v>
+        <v>49.725566374889411</v>
       </c>
       <c r="H33">
-        <v>16.824637442608388</v>
+        <v>22.73628524706481</v>
       </c>
     </row>
     <row r="34" spans="2:8">
@@ -23446,19 +23383,19 @@
         <v>404</v>
       </c>
       <c r="C34">
-        <v>54.059169587861376</v>
+        <v>50.329104893700588</v>
       </c>
       <c r="D34">
-        <v>20.643266624036407</v>
+        <v>23.511924325985657</v>
       </c>
       <c r="F34" t="s">
-        <v>553</v>
+        <v>539</v>
       </c>
       <c r="G34">
-        <v>54.059169587861376</v>
+        <v>50.329104893700588</v>
       </c>
       <c r="H34">
-        <v>20.643266624036407</v>
+        <v>23.511924325985657</v>
       </c>
     </row>
     <row r="35" spans="2:8">
@@ -23466,19 +23403,19 @@
         <v>405</v>
       </c>
       <c r="C35">
-        <v>54.160621229584443</v>
+        <v>49.925997532530509</v>
       </c>
       <c r="D35">
-        <v>16.92764152265681</v>
+        <v>19.974964350935519</v>
       </c>
       <c r="F35" t="s">
-        <v>554</v>
+        <v>540</v>
       </c>
       <c r="G35">
-        <v>54.160621229584443</v>
+        <v>49.925997532530509</v>
       </c>
       <c r="H35">
-        <v>16.92764152265681</v>
+        <v>19.974964350935519</v>
       </c>
     </row>
     <row r="36" spans="2:8">
@@ -23486,19 +23423,19 @@
         <v>406</v>
       </c>
       <c r="C36">
-        <v>53.850966420117743</v>
+        <v>50.373976316407479</v>
       </c>
       <c r="D36">
-        <v>19.007446557812909</v>
+        <v>18.855198827926174</v>
       </c>
       <c r="F36" t="s">
-        <v>555</v>
+        <v>541</v>
       </c>
       <c r="G36">
-        <v>53.850966420117743</v>
+        <v>50.373976316407479</v>
       </c>
       <c r="H36">
-        <v>19.007446557812909</v>
+        <v>18.855198827926174</v>
       </c>
     </row>
     <row r="37" spans="2:8">
@@ -23506,19 +23443,19 @@
         <v>407</v>
       </c>
       <c r="C37">
-        <v>52.430848156657824</v>
+        <v>51.996387905088739</v>
       </c>
       <c r="D37">
-        <v>23.043264145360411</v>
+        <v>18.49109582272952</v>
       </c>
       <c r="F37" t="s">
-        <v>556</v>
+        <v>542</v>
       </c>
       <c r="G37">
-        <v>52.430848156657824</v>
+        <v>51.996387905088739</v>
       </c>
       <c r="H37">
-        <v>23.043264145360411</v>
+        <v>18.49109582272952</v>
       </c>
     </row>
     <row r="38" spans="2:8">
@@ -23526,19 +23463,19 @@
         <v>408</v>
       </c>
       <c r="C38">
-        <v>54.306478182754368</v>
+        <v>52.848851245773041</v>
       </c>
       <c r="D38">
-        <v>22.2025648456056</v>
+        <v>18.672302969332311</v>
       </c>
       <c r="F38" t="s">
-        <v>557</v>
+        <v>543</v>
       </c>
       <c r="G38">
-        <v>54.306478182754368</v>
+        <v>52.848851245773041</v>
       </c>
       <c r="H38">
-        <v>22.2025648456056</v>
+        <v>18.672302969332311</v>
       </c>
     </row>
     <row r="39" spans="2:8">
@@ -23546,19 +23483,19 @@
         <v>409</v>
       </c>
       <c r="C39">
-        <v>53.408286508261966</v>
+        <v>52.463652089533532</v>
       </c>
       <c r="D39">
-        <v>22.619231503504921</v>
+        <v>21.103293415309576</v>
       </c>
       <c r="F39" t="s">
-        <v>558</v>
+        <v>544</v>
       </c>
       <c r="G39">
-        <v>53.408286508261966</v>
+        <v>52.463652089533532</v>
       </c>
       <c r="H39">
-        <v>22.619231503504921</v>
+        <v>21.103293415309576</v>
       </c>
     </row>
     <row r="40" spans="2:8">
@@ -23566,19 +23503,19 @@
         <v>410</v>
       </c>
       <c r="C40">
-        <v>49.725566374889411</v>
+        <v>51.291433003066999</v>
       </c>
       <c r="D40">
-        <v>22.73628524706481</v>
+        <v>20.661910967063164</v>
       </c>
       <c r="F40" t="s">
-        <v>559</v>
+        <v>545</v>
       </c>
       <c r="G40">
-        <v>49.725566374889411</v>
+        <v>51.291433003066999</v>
       </c>
       <c r="H40">
-        <v>22.73628524706481</v>
+        <v>20.661910967063164</v>
       </c>
     </row>
     <row r="41" spans="2:8">
@@ -23586,19 +23523,19 @@
         <v>411</v>
       </c>
       <c r="C41">
-        <v>50.329104893700588</v>
+        <v>51.935870244934229</v>
       </c>
       <c r="D41">
-        <v>23.511924325985657</v>
+        <v>21.901398412958557</v>
       </c>
       <c r="F41" t="s">
-        <v>560</v>
+        <v>546</v>
       </c>
       <c r="G41">
-        <v>50.329104893700588</v>
+        <v>51.935870244934229</v>
       </c>
       <c r="H41">
-        <v>23.511924325985657</v>
+        <v>21.901398412958557</v>
       </c>
     </row>
     <row r="42" spans="2:8">
@@ -23606,19 +23543,19 @@
         <v>412</v>
       </c>
       <c r="C42">
-        <v>49.925997532530509</v>
+        <v>51.945619106835984</v>
       </c>
       <c r="D42">
-        <v>19.974964350935519</v>
+        <v>20.569491805687608</v>
       </c>
       <c r="F42" t="s">
-        <v>561</v>
+        <v>547</v>
       </c>
       <c r="G42">
-        <v>49.925997532530509</v>
+        <v>51.945619106835984</v>
       </c>
       <c r="H42">
-        <v>19.974964350935519</v>
+        <v>20.569491805687608</v>
       </c>
     </row>
     <row r="43" spans="2:8">
@@ -23626,19 +23563,19 @@
         <v>413</v>
       </c>
       <c r="C43">
-        <v>50.373976316407479</v>
+        <v>50.551911719897767</v>
       </c>
       <c r="D43">
-        <v>18.855198827926174</v>
+        <v>21.215073317961568</v>
       </c>
       <c r="F43" t="s">
-        <v>562</v>
+        <v>548</v>
       </c>
       <c r="G43">
-        <v>50.373976316407479</v>
+        <v>50.551911719897767</v>
       </c>
       <c r="H43">
-        <v>18.855198827926174</v>
+        <v>21.215073317961568</v>
       </c>
     </row>
     <row r="44" spans="2:8">
@@ -23646,19 +23583,19 @@
         <v>414</v>
       </c>
       <c r="C44">
-        <v>51.996387905088739</v>
+        <v>52.402780027123931</v>
       </c>
       <c r="D44">
-        <v>18.49109582272952</v>
+        <v>22.221541482666314</v>
       </c>
       <c r="F44" t="s">
-        <v>563</v>
+        <v>549</v>
       </c>
       <c r="G44">
-        <v>51.996387905088739</v>
+        <v>52.402780027123931</v>
       </c>
       <c r="H44">
-        <v>18.49109582272952</v>
+        <v>22.221541482666314</v>
       </c>
     </row>
     <row r="45" spans="2:8">
@@ -23666,19 +23603,19 @@
         <v>415</v>
       </c>
       <c r="C45">
-        <v>52.848851245773041</v>
+        <v>50.221928080120989</v>
       </c>
       <c r="D45">
-        <v>18.672302969332311</v>
+        <v>23.413558137569936</v>
       </c>
       <c r="F45" t="s">
-        <v>564</v>
+        <v>550</v>
       </c>
       <c r="G45">
-        <v>52.848851245773041</v>
+        <v>50.221928080120989</v>
       </c>
       <c r="H45">
-        <v>18.672302969332311</v>
+        <v>23.413558137569936</v>
       </c>
     </row>
     <row r="46" spans="2:8">
@@ -23686,19 +23623,19 @@
         <v>416</v>
       </c>
       <c r="C46">
-        <v>52.463652089533532</v>
+        <v>53.760902274894448</v>
       </c>
       <c r="D46">
-        <v>21.103293415309576</v>
+        <v>22.593353600809184</v>
       </c>
       <c r="F46" t="s">
-        <v>565</v>
+        <v>551</v>
       </c>
       <c r="G46">
-        <v>52.463652089533532</v>
+        <v>53.760902274894448</v>
       </c>
       <c r="H46">
-        <v>21.103293415309576</v>
+        <v>22.593353600809184</v>
       </c>
     </row>
     <row r="47" spans="2:8">
@@ -23706,19 +23643,19 @@
         <v>417</v>
       </c>
       <c r="C47">
-        <v>51.291433003066999</v>
+        <v>52.378757098306828</v>
       </c>
       <c r="D47">
-        <v>20.661910967063164</v>
+        <v>18.692082563317275</v>
       </c>
       <c r="F47" t="s">
-        <v>566</v>
+        <v>552</v>
       </c>
       <c r="G47">
-        <v>51.291433003066999</v>
+        <v>52.378757098306828</v>
       </c>
       <c r="H47">
-        <v>20.661910967063164</v>
+        <v>18.692082563317275</v>
       </c>
     </row>
     <row r="48" spans="2:8">
@@ -23726,19 +23663,19 @@
         <v>418</v>
       </c>
       <c r="C48">
-        <v>51.935870244934229</v>
+        <v>53.14080843144523</v>
       </c>
       <c r="D48">
-        <v>21.901398412958557</v>
+        <v>20.68150354863176</v>
       </c>
       <c r="F48" t="s">
-        <v>567</v>
+        <v>553</v>
       </c>
       <c r="G48">
-        <v>51.935870244934229</v>
+        <v>53.14080843144523</v>
       </c>
       <c r="H48">
-        <v>21.901398412958557</v>
+        <v>20.68150354863176</v>
       </c>
     </row>
     <row r="49" spans="2:8">
@@ -23746,19 +23683,19 @@
         <v>419</v>
       </c>
       <c r="C49">
-        <v>51.945619106835984</v>
+        <v>54.312441674352527</v>
       </c>
       <c r="D49">
-        <v>20.569491805687608</v>
+        <v>21.103188435801304</v>
       </c>
       <c r="F49" t="s">
-        <v>568</v>
+        <v>554</v>
       </c>
       <c r="G49">
-        <v>51.945619106835984</v>
+        <v>54.312441674352527</v>
       </c>
       <c r="H49">
-        <v>20.569491805687608</v>
+        <v>21.103188435801304</v>
       </c>
     </row>
     <row r="50" spans="2:8">
@@ -23766,19 +23703,19 @@
         <v>420</v>
       </c>
       <c r="C50">
-        <v>50.551911719897767</v>
+        <v>53.94247081838023</v>
       </c>
       <c r="D50">
-        <v>21.215073317961568</v>
+        <v>19.258540287803484</v>
       </c>
       <c r="F50" t="s">
-        <v>569</v>
+        <v>555</v>
       </c>
       <c r="G50">
-        <v>50.551911719897767</v>
+        <v>53.94247081838023</v>
       </c>
       <c r="H50">
-        <v>21.215073317961568</v>
+        <v>19.258540287803484</v>
       </c>
     </row>
     <row r="51" spans="2:8">
@@ -23786,19 +23723,19 @@
         <v>421</v>
       </c>
       <c r="C51">
-        <v>52.402780027123931</v>
+        <v>54.161619422062977</v>
       </c>
       <c r="D51">
-        <v>22.221541482666314</v>
+        <v>16.903251720257263</v>
       </c>
       <c r="F51" t="s">
-        <v>570</v>
+        <v>556</v>
       </c>
       <c r="G51">
-        <v>52.402780027123931</v>
+        <v>54.161619422062977</v>
       </c>
       <c r="H51">
-        <v>22.221541482666314</v>
+        <v>16.903251720257263</v>
       </c>
     </row>
     <row r="52" spans="2:8">
@@ -23806,19 +23743,19 @@
         <v>422</v>
       </c>
       <c r="C52">
-        <v>50.221928080120989</v>
+        <v>51.244509727206612</v>
       </c>
       <c r="D52">
-        <v>23.413558137569936</v>
+        <v>15.361927969342226</v>
       </c>
       <c r="F52" t="s">
-        <v>571</v>
+        <v>557</v>
       </c>
       <c r="G52">
-        <v>50.221928080120989</v>
+        <v>51.244509727206612</v>
       </c>
       <c r="H52">
-        <v>23.413558137569936</v>
+        <v>15.361927969342226</v>
       </c>
     </row>
     <row r="53" spans="2:8">
@@ -23826,19 +23763,19 @@
         <v>423</v>
       </c>
       <c r="C53">
-        <v>53.760902274894448</v>
+        <v>52.383060462397033</v>
       </c>
       <c r="D53">
-        <v>22.593353600809184</v>
+        <v>15.026892107180988</v>
       </c>
       <c r="F53" t="s">
-        <v>572</v>
+        <v>558</v>
       </c>
       <c r="G53">
-        <v>53.760902274894448</v>
+        <v>52.383060462397033</v>
       </c>
       <c r="H53">
-        <v>22.593353600809184</v>
+        <v>15.026892107180988</v>
       </c>
     </row>
     <row r="54" spans="2:8">
@@ -23846,19 +23783,19 @@
         <v>424</v>
       </c>
       <c r="C54">
-        <v>52.378757098306828</v>
+        <v>51.541179017177562</v>
       </c>
       <c r="D54">
-        <v>18.692082563317275</v>
+        <v>16.375814143056594</v>
       </c>
       <c r="F54" t="s">
-        <v>573</v>
+        <v>559</v>
       </c>
       <c r="G54">
-        <v>52.378757098306828</v>
+        <v>51.541179017177562</v>
       </c>
       <c r="H54">
-        <v>18.692082563317275</v>
+        <v>16.375814143056594</v>
       </c>
     </row>
     <row r="55" spans="2:8">
@@ -23866,19 +23803,19 @@
         <v>425</v>
       </c>
       <c r="C55">
-        <v>53.14080843144523</v>
+        <v>52.951863842623695</v>
       </c>
       <c r="D55">
-        <v>20.68150354863176</v>
+        <v>16.859888285978002</v>
       </c>
       <c r="F55" t="s">
-        <v>574</v>
+        <v>560</v>
       </c>
       <c r="G55">
-        <v>53.14080843144523</v>
+        <v>52.951863842623695</v>
       </c>
       <c r="H55">
-        <v>20.68150354863176</v>
+        <v>16.859888285978002</v>
       </c>
     </row>
     <row r="56" spans="2:8">
@@ -23886,19 +23823,19 @@
         <v>426</v>
       </c>
       <c r="C56">
-        <v>54.312441674352527</v>
+        <v>49.445868999757508</v>
       </c>
       <c r="D56">
-        <v>21.103188435801304</v>
+        <v>19.826467717110425</v>
       </c>
       <c r="F56" t="s">
-        <v>575</v>
+        <v>561</v>
       </c>
       <c r="G56">
-        <v>54.312441674352527</v>
+        <v>49.445868999757508</v>
       </c>
       <c r="H56">
-        <v>21.103188435801304</v>
+        <v>19.826467717110425</v>
       </c>
     </row>
     <row r="57" spans="2:8">
@@ -23906,19 +23843,19 @@
         <v>427</v>
       </c>
       <c r="C57">
-        <v>53.94247081838023</v>
+        <v>49.445868999757522</v>
       </c>
       <c r="D57">
-        <v>19.258540287803484</v>
+        <v>22.221149843265444</v>
       </c>
       <c r="F57" t="s">
-        <v>576</v>
+        <v>562</v>
       </c>
       <c r="G57">
-        <v>53.94247081838023</v>
+        <v>49.445868999757522</v>
       </c>
       <c r="H57">
-        <v>19.258540287803484</v>
+        <v>22.221149843265444</v>
       </c>
     </row>
     <row r="58" spans="2:8">
@@ -23926,19 +23863,19 @@
         <v>428</v>
       </c>
       <c r="C58">
-        <v>54.161619422062977</v>
+        <v>49.735591777639613</v>
       </c>
       <c r="D58">
-        <v>16.903251720257263</v>
+        <v>21.136931470305012</v>
       </c>
       <c r="F58" t="s">
-        <v>577</v>
+        <v>563</v>
       </c>
       <c r="G58">
-        <v>54.161619422062977</v>
+        <v>49.735591777639613</v>
       </c>
       <c r="H58">
-        <v>16.903251720257263</v>
+        <v>21.136931470305012</v>
       </c>
     </row>
     <row r="59" spans="2:8">
@@ -23946,19 +23883,19 @@
         <v>429</v>
       </c>
       <c r="C59">
-        <v>51.244509727206612</v>
+        <v>50.345189363482064</v>
       </c>
       <c r="D59">
-        <v>15.361927969342226</v>
+        <v>16.733772344126869</v>
       </c>
       <c r="F59" t="s">
-        <v>578</v>
+        <v>564</v>
       </c>
       <c r="G59">
-        <v>51.244509727206612</v>
+        <v>50.345189363482064</v>
       </c>
       <c r="H59">
-        <v>15.361927969342226</v>
+        <v>16.733772344126869</v>
       </c>
     </row>
     <row r="60" spans="2:8">
@@ -23966,19 +23903,19 @@
         <v>430</v>
       </c>
       <c r="C60">
-        <v>52.383060462397033</v>
+        <v>50.203591507323402</v>
       </c>
       <c r="D60">
-        <v>15.026892107180988</v>
+        <v>19.682335745634312</v>
       </c>
       <c r="F60" t="s">
-        <v>579</v>
+        <v>565</v>
       </c>
       <c r="G60">
-        <v>52.383060462397033</v>
+        <v>50.203591507323402</v>
       </c>
       <c r="H60">
-        <v>15.026892107180988</v>
+        <v>19.682335745634312</v>
       </c>
     </row>
     <row r="61" spans="2:8">
@@ -23986,19 +23923,19 @@
         <v>431</v>
       </c>
       <c r="C61">
-        <v>51.541179017177562</v>
+        <v>49.960030388543707</v>
       </c>
       <c r="D61">
-        <v>16.375814143056594</v>
+        <v>18.59892442917592</v>
       </c>
       <c r="F61" t="s">
-        <v>580</v>
+        <v>566</v>
       </c>
       <c r="G61">
-        <v>51.541179017177562</v>
+        <v>49.960030388543707</v>
       </c>
       <c r="H61">
-        <v>16.375814143056594</v>
+        <v>18.59892442917592</v>
       </c>
     </row>
     <row r="62" spans="2:8">
@@ -24006,19 +23943,19 @@
         <v>432</v>
       </c>
       <c r="C62">
-        <v>52.951863842623695</v>
+        <v>54.260443399297102</v>
       </c>
       <c r="D62">
-        <v>16.859888285978002</v>
+        <v>19.270472330221128</v>
       </c>
       <c r="F62" t="s">
-        <v>581</v>
+        <v>567</v>
       </c>
       <c r="G62">
-        <v>52.951863842623695</v>
+        <v>54.260443399297102</v>
       </c>
       <c r="H62">
-        <v>16.859888285978002</v>
+        <v>19.270472330221128</v>
       </c>
     </row>
     <row r="63" spans="2:8">
@@ -24026,19 +23963,19 @@
         <v>433</v>
       </c>
       <c r="C63">
-        <v>49.445868999757508</v>
+        <v>55.159763763021651</v>
       </c>
       <c r="D63">
-        <v>19.826467717110425</v>
+        <v>19.132260930767764</v>
       </c>
       <c r="F63" t="s">
-        <v>582</v>
+        <v>568</v>
       </c>
       <c r="G63">
-        <v>49.445868999757508</v>
+        <v>55.159763763021651</v>
       </c>
       <c r="H63">
-        <v>19.826467717110425</v>
+        <v>19.132260930767764</v>
       </c>
     </row>
     <row r="64" spans="2:8">
@@ -24046,19 +23983,19 @@
         <v>434</v>
       </c>
       <c r="C64">
-        <v>49.445868999757522</v>
+        <v>54.710103581159373</v>
       </c>
       <c r="D64">
-        <v>22.221149843265444</v>
+        <v>19.209642059320888</v>
       </c>
       <c r="F64" t="s">
-        <v>583</v>
+        <v>569</v>
       </c>
       <c r="G64">
-        <v>49.445868999757522</v>
+        <v>54.710103581159373</v>
       </c>
       <c r="H64">
-        <v>22.221149843265444</v>
+        <v>19.209642059320888</v>
       </c>
     </row>
     <row r="65" spans="2:8">
@@ -24066,19 +24003,19 @@
         <v>435</v>
       </c>
       <c r="C65">
-        <v>49.735591777639613</v>
+        <v>55.609423944883922</v>
       </c>
       <c r="D65">
-        <v>21.136931470305012</v>
+        <v>16.941424009640372</v>
       </c>
       <c r="F65" t="s">
-        <v>584</v>
+        <v>570</v>
       </c>
       <c r="G65">
-        <v>49.735591777639613</v>
+        <v>55.609423944883922</v>
       </c>
       <c r="H65">
-        <v>21.136931470305012</v>
+        <v>16.941424009640372</v>
       </c>
     </row>
     <row r="66" spans="2:8">
@@ -24086,19 +24023,19 @@
         <v>436</v>
       </c>
       <c r="C66">
-        <v>50.345189363482064</v>
+        <v>55.609423944883922</v>
       </c>
       <c r="D66">
-        <v>16.733772344126869</v>
+        <v>18.450609737767209</v>
       </c>
       <c r="F66" t="s">
-        <v>585</v>
+        <v>571</v>
       </c>
       <c r="G66">
-        <v>50.345189363482064</v>
+        <v>55.609423944883922</v>
       </c>
       <c r="H66">
-        <v>16.733772344126869</v>
+        <v>18.450609737767209</v>
       </c>
     </row>
     <row r="67" spans="2:8">
@@ -24106,19 +24043,19 @@
         <v>437</v>
       </c>
       <c r="C67">
-        <v>50.203591507323402</v>
+        <v>55.159763763021651</v>
       </c>
       <c r="D67">
-        <v>19.682335745634312</v>
+        <v>17.878339404336558</v>
       </c>
       <c r="F67" t="s">
-        <v>586</v>
+        <v>572</v>
       </c>
       <c r="G67">
-        <v>50.203591507323402</v>
+        <v>55.159763763021651</v>
       </c>
       <c r="H67">
-        <v>19.682335745634312</v>
+        <v>17.878339404336558</v>
       </c>
     </row>
     <row r="68" spans="2:8">
@@ -24126,19 +24063,19 @@
         <v>438</v>
       </c>
       <c r="C68">
-        <v>49.960030388543707</v>
+        <v>54.260443399297102</v>
       </c>
       <c r="D68">
-        <v>18.59892442917592</v>
+        <v>15.473861680498253</v>
       </c>
       <c r="F68" t="s">
-        <v>587</v>
+        <v>573</v>
       </c>
       <c r="G68">
-        <v>49.960030388543707</v>
+        <v>54.260443399297102</v>
       </c>
       <c r="H68">
-        <v>18.59892442917592</v>
+        <v>15.473861680498253</v>
       </c>
     </row>
     <row r="69" spans="2:8">
@@ -24146,19 +24083,19 @@
         <v>439</v>
       </c>
       <c r="C69">
-        <v>54.260443399297102</v>
+        <v>54.71010358115938</v>
       </c>
       <c r="D69">
-        <v>19.270472330221128</v>
+        <v>15.288202232632583</v>
       </c>
       <c r="F69" t="s">
-        <v>588</v>
+        <v>574</v>
       </c>
       <c r="G69">
-        <v>54.260443399297102</v>
+        <v>54.71010358115938</v>
       </c>
       <c r="H69">
-        <v>19.270472330221128</v>
+        <v>15.288202232632583</v>
       </c>
     </row>
     <row r="70" spans="2:8">
@@ -24169,16 +24106,16 @@
         <v>55.159763763021651</v>
       </c>
       <c r="D70">
-        <v>19.132260930767764</v>
+        <v>16.268434622192224</v>
       </c>
       <c r="F70" t="s">
-        <v>589</v>
+        <v>575</v>
       </c>
       <c r="G70">
         <v>55.159763763021651</v>
       </c>
       <c r="H70">
-        <v>19.132260930767764</v>
+        <v>16.268434622192224</v>
       </c>
     </row>
     <row r="71" spans="2:8">
@@ -24189,155 +24126,15 @@
         <v>54.710103581159373</v>
       </c>
       <c r="D71">
-        <v>19.209642059320888</v>
+        <v>16.047850156734548</v>
       </c>
       <c r="F71" t="s">
-        <v>590</v>
+        <v>576</v>
       </c>
       <c r="G71">
         <v>54.710103581159373</v>
       </c>
       <c r="H71">
-        <v>19.209642059320888</v>
-      </c>
-    </row>
-    <row r="72" spans="2:8">
-      <c r="B72" t="s">
-        <v>442</v>
-      </c>
-      <c r="C72">
-        <v>55.609423944883922</v>
-      </c>
-      <c r="D72">
-        <v>16.941424009640372</v>
-      </c>
-      <c r="F72" t="s">
-        <v>591</v>
-      </c>
-      <c r="G72">
-        <v>55.609423944883922</v>
-      </c>
-      <c r="H72">
-        <v>16.941424009640372</v>
-      </c>
-    </row>
-    <row r="73" spans="2:8">
-      <c r="B73" t="s">
-        <v>443</v>
-      </c>
-      <c r="C73">
-        <v>55.609423944883922</v>
-      </c>
-      <c r="D73">
-        <v>18.450609737767209</v>
-      </c>
-      <c r="F73" t="s">
-        <v>592</v>
-      </c>
-      <c r="G73">
-        <v>55.609423944883922</v>
-      </c>
-      <c r="H73">
-        <v>18.450609737767209</v>
-      </c>
-    </row>
-    <row r="74" spans="2:8">
-      <c r="B74" t="s">
-        <v>444</v>
-      </c>
-      <c r="C74">
-        <v>55.159763763021651</v>
-      </c>
-      <c r="D74">
-        <v>17.878339404336558</v>
-      </c>
-      <c r="F74" t="s">
-        <v>593</v>
-      </c>
-      <c r="G74">
-        <v>55.159763763021651</v>
-      </c>
-      <c r="H74">
-        <v>17.878339404336558</v>
-      </c>
-    </row>
-    <row r="75" spans="2:8">
-      <c r="B75" t="s">
-        <v>445</v>
-      </c>
-      <c r="C75">
-        <v>54.260443399297102</v>
-      </c>
-      <c r="D75">
-        <v>15.473861680498253</v>
-      </c>
-      <c r="F75" t="s">
-        <v>594</v>
-      </c>
-      <c r="G75">
-        <v>54.260443399297102</v>
-      </c>
-      <c r="H75">
-        <v>15.473861680498253</v>
-      </c>
-    </row>
-    <row r="76" spans="2:8">
-      <c r="B76" t="s">
-        <v>446</v>
-      </c>
-      <c r="C76">
-        <v>54.71010358115938</v>
-      </c>
-      <c r="D76">
-        <v>15.288202232632583</v>
-      </c>
-      <c r="F76" t="s">
-        <v>595</v>
-      </c>
-      <c r="G76">
-        <v>54.71010358115938</v>
-      </c>
-      <c r="H76">
-        <v>15.288202232632583</v>
-      </c>
-    </row>
-    <row r="77" spans="2:8">
-      <c r="B77" t="s">
-        <v>447</v>
-      </c>
-      <c r="C77">
-        <v>55.159763763021651</v>
-      </c>
-      <c r="D77">
-        <v>16.268434622192224</v>
-      </c>
-      <c r="F77" t="s">
-        <v>596</v>
-      </c>
-      <c r="G77">
-        <v>55.159763763021651</v>
-      </c>
-      <c r="H77">
-        <v>16.268434622192224</v>
-      </c>
-    </row>
-    <row r="78" spans="2:8">
-      <c r="B78" t="s">
-        <v>448</v>
-      </c>
-      <c r="C78">
-        <v>54.710103581159373</v>
-      </c>
-      <c r="D78">
-        <v>16.047850156734548</v>
-      </c>
-      <c r="F78" t="s">
-        <v>597</v>
-      </c>
-      <c r="G78">
-        <v>54.710103581159373</v>
-      </c>
-      <c r="H78">
         <v>16.047850156734548</v>
       </c>
     </row>
@@ -24347,8 +24144,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73462742-1544-4D58-977F-CCB49A4C9ABC}">
-  <dimension ref="B9:L78"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EE06E89-FC1C-428A-9A36-8602FB51D88A}">
+  <dimension ref="B9:L71"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:12">
@@ -24405,19 +24202,19 @@
         <v>381</v>
       </c>
       <c r="G11" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H11" t="s">
-        <v>450</v>
+        <v>443</v>
       </c>
       <c r="J11" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K11" t="s">
-        <v>459</v>
+        <v>452</v>
       </c>
       <c r="L11" t="s">
-        <v>459</v>
+        <v>452</v>
       </c>
     </row>
     <row r="12" spans="2:12">
@@ -24434,19 +24231,19 @@
         <v>382</v>
       </c>
       <c r="G12" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H12" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
       <c r="J12" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K12" t="s">
-        <v>460</v>
+        <v>453</v>
       </c>
       <c r="L12" t="s">
-        <v>460</v>
+        <v>453</v>
       </c>
     </row>
     <row r="13" spans="2:12">
@@ -24463,19 +24260,19 @@
         <v>383</v>
       </c>
       <c r="G13" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H13" t="s">
+        <v>445</v>
+      </c>
+      <c r="J13" t="s">
         <v>451</v>
       </c>
-      <c r="J13" t="s">
-        <v>458</v>
-      </c>
       <c r="K13" t="s">
-        <v>461</v>
+        <v>454</v>
       </c>
       <c r="L13" t="s">
-        <v>461</v>
+        <v>454</v>
       </c>
     </row>
     <row r="14" spans="2:12">
@@ -24492,19 +24289,19 @@
         <v>384</v>
       </c>
       <c r="G14" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H14" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="J14" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K14" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
       <c r="L14" t="s">
-        <v>462</v>
+        <v>455</v>
       </c>
     </row>
     <row r="15" spans="2:12">
@@ -24521,19 +24318,19 @@
         <v>385</v>
       </c>
       <c r="G15" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H15" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="J15" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K15" t="s">
-        <v>463</v>
+        <v>456</v>
       </c>
       <c r="L15" t="s">
-        <v>463</v>
+        <v>456</v>
       </c>
     </row>
     <row r="16" spans="2:12">
@@ -24550,19 +24347,19 @@
         <v>386</v>
       </c>
       <c r="G16" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H16" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="J16" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K16" t="s">
-        <v>464</v>
+        <v>457</v>
       </c>
       <c r="L16" t="s">
-        <v>464</v>
+        <v>457</v>
       </c>
     </row>
     <row r="17" spans="2:12">
@@ -24579,19 +24376,19 @@
         <v>387</v>
       </c>
       <c r="G17" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H17" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="J17" t="s">
+        <v>451</v>
+      </c>
+      <c r="K17" t="s">
         <v>458</v>
       </c>
-      <c r="K17" t="s">
-        <v>465</v>
-      </c>
       <c r="L17" t="s">
-        <v>465</v>
+        <v>458</v>
       </c>
     </row>
     <row r="18" spans="2:12">
@@ -24608,19 +24405,19 @@
         <v>388</v>
       </c>
       <c r="G18" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H18" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="J18" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K18" t="s">
-        <v>466</v>
+        <v>459</v>
       </c>
       <c r="L18" t="s">
-        <v>466</v>
+        <v>459</v>
       </c>
     </row>
     <row r="19" spans="2:12">
@@ -24637,19 +24434,19 @@
         <v>389</v>
       </c>
       <c r="G19" t="s">
+        <v>442</v>
+      </c>
+      <c r="H19" t="s">
         <v>449</v>
       </c>
-      <c r="H19" t="s">
+      <c r="J19" t="s">
         <v>451</v>
       </c>
-      <c r="J19" t="s">
-        <v>458</v>
-      </c>
       <c r="K19" t="s">
-        <v>467</v>
+        <v>460</v>
       </c>
       <c r="L19" t="s">
-        <v>467</v>
+        <v>460</v>
       </c>
     </row>
     <row r="20" spans="2:12">
@@ -24666,19 +24463,19 @@
         <v>390</v>
       </c>
       <c r="G20" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H20" t="s">
-        <v>450</v>
+        <v>445</v>
       </c>
       <c r="J20" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K20" t="s">
-        <v>468</v>
+        <v>461</v>
       </c>
       <c r="L20" t="s">
-        <v>468</v>
+        <v>461</v>
       </c>
     </row>
     <row r="21" spans="2:12">
@@ -24695,19 +24492,19 @@
         <v>391</v>
       </c>
       <c r="G21" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H21" t="s">
-        <v>450</v>
+        <v>445</v>
       </c>
       <c r="J21" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K21" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
       <c r="L21" t="s">
-        <v>469</v>
+        <v>462</v>
       </c>
     </row>
     <row r="22" spans="2:12">
@@ -24724,19 +24521,19 @@
         <v>392</v>
       </c>
       <c r="G22" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H22" t="s">
-        <v>455</v>
+        <v>444</v>
       </c>
       <c r="J22" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K22" t="s">
-        <v>470</v>
+        <v>463</v>
       </c>
       <c r="L22" t="s">
-        <v>470</v>
+        <v>463</v>
       </c>
     </row>
     <row r="23" spans="2:12">
@@ -24753,19 +24550,19 @@
         <v>393</v>
       </c>
       <c r="G23" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H23" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="J23" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K23" t="s">
-        <v>471</v>
+        <v>464</v>
       </c>
       <c r="L23" t="s">
-        <v>471</v>
+        <v>464</v>
       </c>
     </row>
     <row r="24" spans="2:12">
@@ -24782,19 +24579,19 @@
         <v>394</v>
       </c>
       <c r="G24" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H24" t="s">
-        <v>456</v>
+        <v>446</v>
       </c>
       <c r="J24" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K24" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
       <c r="L24" t="s">
-        <v>472</v>
+        <v>465</v>
       </c>
     </row>
     <row r="25" spans="2:12">
@@ -24811,19 +24608,19 @@
         <v>395</v>
       </c>
       <c r="G25" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H25" t="s">
-        <v>452</v>
+        <v>444</v>
       </c>
       <c r="J25" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K25" t="s">
-        <v>473</v>
+        <v>466</v>
       </c>
       <c r="L25" t="s">
-        <v>473</v>
+        <v>466</v>
       </c>
     </row>
     <row r="26" spans="2:12">
@@ -24840,19 +24637,19 @@
         <v>396</v>
       </c>
       <c r="G26" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H26" t="s">
-        <v>456</v>
+        <v>444</v>
       </c>
       <c r="J26" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K26" t="s">
-        <v>474</v>
+        <v>467</v>
       </c>
       <c r="L26" t="s">
-        <v>474</v>
+        <v>467</v>
       </c>
     </row>
     <row r="27" spans="2:12">
@@ -24869,19 +24666,19 @@
         <v>397</v>
       </c>
       <c r="G27" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H27" t="s">
-        <v>456</v>
+        <v>445</v>
       </c>
       <c r="J27" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K27" t="s">
-        <v>475</v>
+        <v>468</v>
       </c>
       <c r="L27" t="s">
-        <v>475</v>
+        <v>468</v>
       </c>
     </row>
     <row r="28" spans="2:12">
@@ -24898,19 +24695,19 @@
         <v>398</v>
       </c>
       <c r="G28" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H28" t="s">
-        <v>456</v>
+        <v>445</v>
       </c>
       <c r="J28" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K28" t="s">
-        <v>476</v>
+        <v>469</v>
       </c>
       <c r="L28" t="s">
-        <v>476</v>
+        <v>469</v>
       </c>
     </row>
     <row r="29" spans="2:12">
@@ -24927,19 +24724,19 @@
         <v>399</v>
       </c>
       <c r="G29" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H29" t="s">
-        <v>454</v>
+        <v>445</v>
       </c>
       <c r="J29" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K29" t="s">
-        <v>477</v>
+        <v>470</v>
       </c>
       <c r="L29" t="s">
-        <v>477</v>
+        <v>470</v>
       </c>
     </row>
     <row r="30" spans="2:12">
@@ -24956,19 +24753,19 @@
         <v>400</v>
       </c>
       <c r="G30" t="s">
+        <v>442</v>
+      </c>
+      <c r="H30" t="s">
         <v>449</v>
       </c>
-      <c r="H30" t="s">
+      <c r="J30" t="s">
         <v>451</v>
       </c>
-      <c r="J30" t="s">
-        <v>458</v>
-      </c>
       <c r="K30" t="s">
-        <v>478</v>
+        <v>471</v>
       </c>
       <c r="L30" t="s">
-        <v>478</v>
+        <v>471</v>
       </c>
     </row>
     <row r="31" spans="2:12">
@@ -24985,19 +24782,19 @@
         <v>401</v>
       </c>
       <c r="G31" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H31" t="s">
+        <v>445</v>
+      </c>
+      <c r="J31" t="s">
         <v>451</v>
       </c>
-      <c r="J31" t="s">
-        <v>458</v>
-      </c>
       <c r="K31" t="s">
-        <v>479</v>
+        <v>472</v>
       </c>
       <c r="L31" t="s">
-        <v>479</v>
+        <v>472</v>
       </c>
     </row>
     <row r="32" spans="2:12">
@@ -25014,19 +24811,19 @@
         <v>402</v>
       </c>
       <c r="G32" t="s">
+        <v>442</v>
+      </c>
+      <c r="H32" t="s">
         <v>449</v>
       </c>
-      <c r="H32" t="s">
-        <v>454</v>
-      </c>
       <c r="J32" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K32" t="s">
-        <v>480</v>
+        <v>473</v>
       </c>
       <c r="L32" t="s">
-        <v>480</v>
+        <v>473</v>
       </c>
     </row>
     <row r="33" spans="2:12">
@@ -25043,19 +24840,19 @@
         <v>403</v>
       </c>
       <c r="G33" t="s">
+        <v>442</v>
+      </c>
+      <c r="H33" t="s">
         <v>449</v>
       </c>
-      <c r="H33" t="s">
-        <v>454</v>
-      </c>
       <c r="J33" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K33" t="s">
-        <v>481</v>
+        <v>474</v>
       </c>
       <c r="L33" t="s">
-        <v>481</v>
+        <v>474</v>
       </c>
     </row>
     <row r="34" spans="2:12">
@@ -25072,19 +24869,19 @@
         <v>404</v>
       </c>
       <c r="G34" t="s">
+        <v>442</v>
+      </c>
+      <c r="H34" t="s">
         <v>449</v>
       </c>
-      <c r="H34" t="s">
-        <v>452</v>
-      </c>
       <c r="J34" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K34" t="s">
-        <v>482</v>
+        <v>475</v>
       </c>
       <c r="L34" t="s">
-        <v>482</v>
+        <v>475</v>
       </c>
     </row>
     <row r="35" spans="2:12">
@@ -25101,19 +24898,19 @@
         <v>405</v>
       </c>
       <c r="G35" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H35" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="J35" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K35" t="s">
-        <v>483</v>
+        <v>476</v>
       </c>
       <c r="L35" t="s">
-        <v>483</v>
+        <v>476</v>
       </c>
     </row>
     <row r="36" spans="2:12">
@@ -25130,19 +24927,19 @@
         <v>406</v>
       </c>
       <c r="G36" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H36" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="J36" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K36" t="s">
-        <v>484</v>
+        <v>477</v>
       </c>
       <c r="L36" t="s">
-        <v>484</v>
+        <v>477</v>
       </c>
     </row>
     <row r="37" spans="2:12">
@@ -25159,19 +24956,19 @@
         <v>407</v>
       </c>
       <c r="G37" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H37" t="s">
-        <v>456</v>
+        <v>444</v>
       </c>
       <c r="J37" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K37" t="s">
-        <v>485</v>
+        <v>478</v>
       </c>
       <c r="L37" t="s">
-        <v>485</v>
+        <v>478</v>
       </c>
     </row>
     <row r="38" spans="2:12">
@@ -25188,19 +24985,19 @@
         <v>408</v>
       </c>
       <c r="G38" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H38" t="s">
-        <v>452</v>
+        <v>445</v>
       </c>
       <c r="J38" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K38" t="s">
-        <v>486</v>
+        <v>479</v>
       </c>
       <c r="L38" t="s">
-        <v>486</v>
+        <v>479</v>
       </c>
     </row>
     <row r="39" spans="2:12">
@@ -25217,19 +25014,19 @@
         <v>409</v>
       </c>
       <c r="G39" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H39" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="J39" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K39" t="s">
-        <v>487</v>
+        <v>480</v>
       </c>
       <c r="L39" t="s">
-        <v>487</v>
+        <v>480</v>
       </c>
     </row>
     <row r="40" spans="2:12">
@@ -25246,19 +25043,19 @@
         <v>410</v>
       </c>
       <c r="G40" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H40" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="J40" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K40" t="s">
-        <v>488</v>
+        <v>481</v>
       </c>
       <c r="L40" t="s">
-        <v>488</v>
+        <v>481</v>
       </c>
     </row>
     <row r="41" spans="2:12">
@@ -25275,19 +25072,19 @@
         <v>411</v>
       </c>
       <c r="G41" t="s">
+        <v>442</v>
+      </c>
+      <c r="H41" t="s">
         <v>449</v>
       </c>
-      <c r="H41" t="s">
-        <v>456</v>
-      </c>
       <c r="J41" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K41" t="s">
-        <v>489</v>
+        <v>482</v>
       </c>
       <c r="L41" t="s">
-        <v>489</v>
+        <v>482</v>
       </c>
     </row>
     <row r="42" spans="2:12">
@@ -25304,19 +25101,19 @@
         <v>412</v>
       </c>
       <c r="G42" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H42" t="s">
-        <v>450</v>
+        <v>443</v>
       </c>
       <c r="J42" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K42" t="s">
-        <v>490</v>
+        <v>483</v>
       </c>
       <c r="L42" t="s">
-        <v>490</v>
+        <v>483</v>
       </c>
     </row>
     <row r="43" spans="2:12">
@@ -25333,19 +25130,19 @@
         <v>413</v>
       </c>
       <c r="G43" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H43" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="J43" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K43" t="s">
-        <v>491</v>
+        <v>484</v>
       </c>
       <c r="L43" t="s">
-        <v>491</v>
+        <v>484</v>
       </c>
     </row>
     <row r="44" spans="2:12">
@@ -25362,19 +25159,19 @@
         <v>414</v>
       </c>
       <c r="G44" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H44" t="s">
-        <v>454</v>
+        <v>443</v>
       </c>
       <c r="J44" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K44" t="s">
-        <v>492</v>
+        <v>485</v>
       </c>
       <c r="L44" t="s">
-        <v>492</v>
+        <v>485</v>
       </c>
     </row>
     <row r="45" spans="2:12">
@@ -25391,19 +25188,19 @@
         <v>415</v>
       </c>
       <c r="G45" t="s">
+        <v>442</v>
+      </c>
+      <c r="H45" t="s">
         <v>449</v>
       </c>
-      <c r="H45" t="s">
-        <v>452</v>
-      </c>
       <c r="J45" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K45" t="s">
-        <v>493</v>
+        <v>486</v>
       </c>
       <c r="L45" t="s">
-        <v>493</v>
+        <v>486</v>
       </c>
     </row>
     <row r="46" spans="2:12">
@@ -25420,19 +25217,19 @@
         <v>416</v>
       </c>
       <c r="G46" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H46" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="J46" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K46" t="s">
-        <v>494</v>
+        <v>487</v>
       </c>
       <c r="L46" t="s">
-        <v>494</v>
+        <v>487</v>
       </c>
     </row>
     <row r="47" spans="2:12">
@@ -25449,19 +25246,19 @@
         <v>417</v>
       </c>
       <c r="G47" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H47" t="s">
-        <v>453</v>
+        <v>444</v>
       </c>
       <c r="J47" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K47" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="L47" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
     </row>
     <row r="48" spans="2:12">
@@ -25478,19 +25275,19 @@
         <v>418</v>
       </c>
       <c r="G48" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H48" t="s">
-        <v>456</v>
+        <v>443</v>
       </c>
       <c r="J48" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K48" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
       <c r="L48" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
     </row>
     <row r="49" spans="2:12">
@@ -25507,19 +25304,19 @@
         <v>419</v>
       </c>
       <c r="G49" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H49" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="J49" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K49" t="s">
-        <v>497</v>
+        <v>490</v>
       </c>
       <c r="L49" t="s">
-        <v>497</v>
+        <v>490</v>
       </c>
     </row>
     <row r="50" spans="2:12">
@@ -25536,19 +25333,19 @@
         <v>420</v>
       </c>
       <c r="G50" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H50" t="s">
-        <v>455</v>
+        <v>445</v>
       </c>
       <c r="J50" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K50" t="s">
-        <v>498</v>
+        <v>491</v>
       </c>
       <c r="L50" t="s">
-        <v>498</v>
+        <v>491</v>
       </c>
     </row>
     <row r="51" spans="2:12">
@@ -25565,19 +25362,19 @@
         <v>421</v>
       </c>
       <c r="G51" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H51" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="J51" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K51" t="s">
-        <v>499</v>
+        <v>492</v>
       </c>
       <c r="L51" t="s">
-        <v>499</v>
+        <v>492</v>
       </c>
     </row>
     <row r="52" spans="2:12">
@@ -25594,19 +25391,19 @@
         <v>422</v>
       </c>
       <c r="G52" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H52" t="s">
-        <v>456</v>
+        <v>446</v>
       </c>
       <c r="J52" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K52" t="s">
-        <v>500</v>
+        <v>493</v>
       </c>
       <c r="L52" t="s">
-        <v>500</v>
+        <v>493</v>
       </c>
     </row>
     <row r="53" spans="2:12">
@@ -25623,19 +25420,19 @@
         <v>423</v>
       </c>
       <c r="G53" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H53" t="s">
-        <v>452</v>
+        <v>444</v>
       </c>
       <c r="J53" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K53" t="s">
-        <v>501</v>
+        <v>494</v>
       </c>
       <c r="L53" t="s">
-        <v>501</v>
+        <v>494</v>
       </c>
     </row>
     <row r="54" spans="2:12">
@@ -25652,19 +25449,19 @@
         <v>424</v>
       </c>
       <c r="G54" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H54" t="s">
-        <v>454</v>
+        <v>446</v>
       </c>
       <c r="J54" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K54" t="s">
-        <v>502</v>
+        <v>495</v>
       </c>
       <c r="L54" t="s">
-        <v>502</v>
+        <v>495</v>
       </c>
     </row>
     <row r="55" spans="2:12">
@@ -25681,19 +25478,19 @@
         <v>425</v>
       </c>
       <c r="G55" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H55" t="s">
-        <v>453</v>
+        <v>444</v>
       </c>
       <c r="J55" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K55" t="s">
-        <v>503</v>
+        <v>496</v>
       </c>
       <c r="L55" t="s">
-        <v>503</v>
+        <v>496</v>
       </c>
     </row>
     <row r="56" spans="2:12">
@@ -25710,19 +25507,19 @@
         <v>426</v>
       </c>
       <c r="G56" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H56" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="J56" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K56" t="s">
-        <v>504</v>
+        <v>497</v>
       </c>
       <c r="L56" t="s">
-        <v>504</v>
+        <v>497</v>
       </c>
     </row>
     <row r="57" spans="2:12">
@@ -25739,19 +25536,19 @@
         <v>427</v>
       </c>
       <c r="G57" t="s">
+        <v>442</v>
+      </c>
+      <c r="H57" t="s">
         <v>449</v>
       </c>
-      <c r="H57" t="s">
-        <v>452</v>
-      </c>
       <c r="J57" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K57" t="s">
-        <v>505</v>
+        <v>498</v>
       </c>
       <c r="L57" t="s">
-        <v>505</v>
+        <v>498</v>
       </c>
     </row>
     <row r="58" spans="2:12">
@@ -25768,19 +25565,19 @@
         <v>428</v>
       </c>
       <c r="G58" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H58" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="J58" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K58" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
       <c r="L58" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
     </row>
     <row r="59" spans="2:12">
@@ -25797,19 +25594,19 @@
         <v>429</v>
       </c>
       <c r="G59" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H59" t="s">
+        <v>446</v>
+      </c>
+      <c r="J59" t="s">
         <v>451</v>
       </c>
-      <c r="J59" t="s">
-        <v>458</v>
-      </c>
       <c r="K59" t="s">
-        <v>507</v>
+        <v>500</v>
       </c>
       <c r="L59" t="s">
-        <v>507</v>
+        <v>500</v>
       </c>
     </row>
     <row r="60" spans="2:12">
@@ -25826,19 +25623,19 @@
         <v>430</v>
       </c>
       <c r="G60" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H60" t="s">
-        <v>454</v>
+        <v>447</v>
       </c>
       <c r="J60" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K60" t="s">
-        <v>508</v>
+        <v>501</v>
       </c>
       <c r="L60" t="s">
-        <v>508</v>
+        <v>501</v>
       </c>
     </row>
     <row r="61" spans="2:12">
@@ -25855,19 +25652,19 @@
         <v>431</v>
       </c>
       <c r="G61" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H61" t="s">
+        <v>447</v>
+      </c>
+      <c r="J61" t="s">
         <v>451</v>
       </c>
-      <c r="J61" t="s">
-        <v>458</v>
-      </c>
       <c r="K61" t="s">
-        <v>509</v>
+        <v>502</v>
       </c>
       <c r="L61" t="s">
-        <v>509</v>
+        <v>502</v>
       </c>
     </row>
     <row r="62" spans="2:12">
@@ -25884,19 +25681,19 @@
         <v>432</v>
       </c>
       <c r="G62" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H62" t="s">
-        <v>454</v>
+        <v>445</v>
       </c>
       <c r="J62" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K62" t="s">
-        <v>510</v>
+        <v>503</v>
       </c>
       <c r="L62" t="s">
-        <v>510</v>
+        <v>503</v>
       </c>
     </row>
     <row r="63" spans="2:12">
@@ -25913,19 +25710,19 @@
         <v>433</v>
       </c>
       <c r="G63" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H63" t="s">
         <v>450</v>
       </c>
       <c r="J63" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K63" t="s">
-        <v>511</v>
+        <v>504</v>
       </c>
       <c r="L63" t="s">
-        <v>511</v>
+        <v>504</v>
       </c>
     </row>
     <row r="64" spans="2:12">
@@ -25942,19 +25739,19 @@
         <v>434</v>
       </c>
       <c r="G64" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H64" t="s">
-        <v>456</v>
+        <v>450</v>
       </c>
       <c r="J64" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K64" t="s">
-        <v>512</v>
+        <v>505</v>
       </c>
       <c r="L64" t="s">
-        <v>512</v>
+        <v>505</v>
       </c>
     </row>
     <row r="65" spans="2:12">
@@ -25971,19 +25768,19 @@
         <v>435</v>
       </c>
       <c r="G65" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H65" t="s">
         <v>450</v>
       </c>
       <c r="J65" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K65" t="s">
-        <v>513</v>
+        <v>506</v>
       </c>
       <c r="L65" t="s">
-        <v>513</v>
+        <v>506</v>
       </c>
     </row>
     <row r="66" spans="2:12">
@@ -26000,19 +25797,19 @@
         <v>436</v>
       </c>
       <c r="G66" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H66" t="s">
+        <v>450</v>
+      </c>
+      <c r="J66" t="s">
         <v>451</v>
       </c>
-      <c r="J66" t="s">
-        <v>458</v>
-      </c>
       <c r="K66" t="s">
-        <v>514</v>
+        <v>507</v>
       </c>
       <c r="L66" t="s">
-        <v>514</v>
+        <v>507</v>
       </c>
     </row>
     <row r="67" spans="2:12">
@@ -26029,19 +25826,19 @@
         <v>437</v>
       </c>
       <c r="G67" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H67" t="s">
         <v>450</v>
       </c>
       <c r="J67" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K67" t="s">
-        <v>515</v>
+        <v>508</v>
       </c>
       <c r="L67" t="s">
-        <v>515</v>
+        <v>508</v>
       </c>
     </row>
     <row r="68" spans="2:12">
@@ -26058,19 +25855,19 @@
         <v>438</v>
       </c>
       <c r="G68" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H68" t="s">
         <v>450</v>
       </c>
       <c r="J68" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K68" t="s">
-        <v>516</v>
+        <v>509</v>
       </c>
       <c r="L68" t="s">
-        <v>516</v>
+        <v>509</v>
       </c>
     </row>
     <row r="69" spans="2:12">
@@ -26087,19 +25884,19 @@
         <v>439</v>
       </c>
       <c r="G69" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H69" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="J69" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K69" t="s">
-        <v>517</v>
+        <v>510</v>
       </c>
       <c r="L69" t="s">
-        <v>517</v>
+        <v>510</v>
       </c>
     </row>
     <row r="70" spans="2:12">
@@ -26116,19 +25913,19 @@
         <v>440</v>
       </c>
       <c r="G70" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H70" t="s">
-        <v>457</v>
+        <v>450</v>
       </c>
       <c r="J70" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K70" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="L70" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
     </row>
     <row r="71" spans="2:12">
@@ -26145,222 +25942,19 @@
         <v>441</v>
       </c>
       <c r="G71" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H71" t="s">
-        <v>457</v>
+        <v>450</v>
       </c>
       <c r="J71" t="s">
-        <v>458</v>
+        <v>451</v>
       </c>
       <c r="K71" t="s">
-        <v>519</v>
+        <v>512</v>
       </c>
       <c r="L71" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="72" spans="2:12">
-      <c r="B72" t="s">
-        <v>380</v>
-      </c>
-      <c r="C72" t="s">
-        <v>442</v>
-      </c>
-      <c r="D72" t="s">
-        <v>442</v>
-      </c>
-      <c r="F72" t="s">
-        <v>442</v>
-      </c>
-      <c r="G72" t="s">
-        <v>449</v>
-      </c>
-      <c r="H72" t="s">
-        <v>457</v>
-      </c>
-      <c r="J72" t="s">
-        <v>458</v>
-      </c>
-      <c r="K72" t="s">
-        <v>520</v>
-      </c>
-      <c r="L72" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="73" spans="2:12">
-      <c r="B73" t="s">
-        <v>380</v>
-      </c>
-      <c r="C73" t="s">
-        <v>443</v>
-      </c>
-      <c r="D73" t="s">
-        <v>443</v>
-      </c>
-      <c r="F73" t="s">
-        <v>443</v>
-      </c>
-      <c r="G73" t="s">
-        <v>449</v>
-      </c>
-      <c r="H73" t="s">
-        <v>457</v>
-      </c>
-      <c r="J73" t="s">
-        <v>458</v>
-      </c>
-      <c r="K73" t="s">
-        <v>521</v>
-      </c>
-      <c r="L73" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="74" spans="2:12">
-      <c r="B74" t="s">
-        <v>380</v>
-      </c>
-      <c r="C74" t="s">
-        <v>444</v>
-      </c>
-      <c r="D74" t="s">
-        <v>444</v>
-      </c>
-      <c r="F74" t="s">
-        <v>444</v>
-      </c>
-      <c r="G74" t="s">
-        <v>449</v>
-      </c>
-      <c r="H74" t="s">
-        <v>457</v>
-      </c>
-      <c r="J74" t="s">
-        <v>458</v>
-      </c>
-      <c r="K74" t="s">
-        <v>522</v>
-      </c>
-      <c r="L74" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="75" spans="2:12">
-      <c r="B75" t="s">
-        <v>380</v>
-      </c>
-      <c r="C75" t="s">
-        <v>445</v>
-      </c>
-      <c r="D75" t="s">
-        <v>445</v>
-      </c>
-      <c r="F75" t="s">
-        <v>445</v>
-      </c>
-      <c r="G75" t="s">
-        <v>449</v>
-      </c>
-      <c r="H75" t="s">
-        <v>457</v>
-      </c>
-      <c r="J75" t="s">
-        <v>458</v>
-      </c>
-      <c r="K75" t="s">
-        <v>523</v>
-      </c>
-      <c r="L75" t="s">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="76" spans="2:12">
-      <c r="B76" t="s">
-        <v>380</v>
-      </c>
-      <c r="C76" t="s">
-        <v>446</v>
-      </c>
-      <c r="D76" t="s">
-        <v>446</v>
-      </c>
-      <c r="F76" t="s">
-        <v>446</v>
-      </c>
-      <c r="G76" t="s">
-        <v>449</v>
-      </c>
-      <c r="H76" t="s">
-        <v>457</v>
-      </c>
-      <c r="J76" t="s">
-        <v>458</v>
-      </c>
-      <c r="K76" t="s">
-        <v>524</v>
-      </c>
-      <c r="L76" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="77" spans="2:12">
-      <c r="B77" t="s">
-        <v>380</v>
-      </c>
-      <c r="C77" t="s">
-        <v>447</v>
-      </c>
-      <c r="D77" t="s">
-        <v>447</v>
-      </c>
-      <c r="F77" t="s">
-        <v>447</v>
-      </c>
-      <c r="G77" t="s">
-        <v>449</v>
-      </c>
-      <c r="H77" t="s">
-        <v>457</v>
-      </c>
-      <c r="J77" t="s">
-        <v>458</v>
-      </c>
-      <c r="K77" t="s">
-        <v>525</v>
-      </c>
-      <c r="L77" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="78" spans="2:12">
-      <c r="B78" t="s">
-        <v>380</v>
-      </c>
-      <c r="C78" t="s">
-        <v>448</v>
-      </c>
-      <c r="D78" t="s">
-        <v>448</v>
-      </c>
-      <c r="F78" t="s">
-        <v>448</v>
-      </c>
-      <c r="G78" t="s">
-        <v>449</v>
-      </c>
-      <c r="H78" t="s">
-        <v>457</v>
-      </c>
-      <c r="J78" t="s">
-        <v>458</v>
-      </c>
-      <c r="K78" t="s">
-        <v>526</v>
-      </c>
-      <c r="L78" t="s">
-        <v>526</v>
+        <v>512</v>
       </c>
     </row>
   </sheetData>

</xml_diff>